<commit_message>
Adding Communcation md file
</commit_message>
<xml_diff>
--- a/Progress.xlsx
+++ b/Progress.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\learnings\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07EE55A8-B93A-4B0B-BF1F-ED286EB25D88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,9 +24,136 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="35">
+  <si>
+    <t>ENGLISH</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>FRONTEND</t>
+  </si>
+  <si>
+    <t>DSA/JAVA</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>TIME</t>
+  </si>
+  <si>
+    <t>PLAN</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>REMARKS</t>
+  </si>
+  <si>
+    <t>PROGRESS                          Start date: 22/7/26</t>
+  </si>
+  <si>
+    <t>7 to 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 to 9 </t>
+  </si>
+  <si>
+    <t>9 to 10</t>
+  </si>
+  <si>
+    <t>10 to 11</t>
+  </si>
+  <si>
+    <t>11 to 12</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>25/7/26</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>26/7/26</t>
+  </si>
+  <si>
+    <t>Git basic commands</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Others</t>
+  </si>
+  <si>
+    <t>Learn basics in Claude code, 
+  need to complete 1 hour youtube video</t>
+  </si>
+  <si>
+    <t>Need to complete balance 1.5 hours of videos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day time
+ spent
+3 hours
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Need to complete claude code 3.5 hour video   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Need to complete 1 hour claude code course - total time 3.5 hour video  </t>
+  </si>
+  <si>
+    <t>Communication practice</t>
+  </si>
+  <si>
+    <t>9.30 to 10.30</t>
+  </si>
+  <si>
+    <t>10.30  to 11</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">45 minutes studied but repeated videos only so </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="6" tint="0.79998168889431442"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No progress</t>
+    </r>
+  </si>
+  <si>
+    <t>22 to 24 React</t>
+  </si>
+  <si>
+    <t>Completed 45 minutes</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +161,75 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="6" tint="0.79998168889431442"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +244,55 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +572,445 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="10.36328125" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="35.08984375" customWidth="1"/>
+    <col min="5" max="5" width="18.90625" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="11"/>
+      <c r="B1" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="14"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+    </row>
+    <row r="11" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="16"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="14"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="1"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="1"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="1"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="1"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="14"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="1"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="1"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="1"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="1"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="1"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="14"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="1"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="1"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="1"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="1"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="1"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="14"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="A5:A9"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A11:A16"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A24:A28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="B5:B9"/>
+    <mergeCell ref="B11:B16"/>
+    <mergeCell ref="B18:B22"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>